<commit_message>
Add easier-to-close prospect sheet (60 businesses, 5 niches)
New Fáciles sheet ranked by ease of close, with WhatsApp as primary
contact, plus FACILES.md reading copy and summary block.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YJJzdLzinEMQwmiWK84eGj
</commit_message>
<xml_diff>
--- a/outreach/prospectos-panama.xlsx
+++ b/outreach/prospectos-panama.xlsx
@@ -8,11 +8,13 @@
   </bookViews>
   <sheets>
     <sheet name="Prospectos" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Resumen" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Cómo usar" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Fáciles" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Resumen" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Cómo usar" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Prospectos'!$A$1:$P$63</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Fáciles'!$A$1:$P$61</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -24,7 +26,7 @@
     <numFmt numFmtId="164" formatCode="DD/MM/YYYY"/>
     <numFmt numFmtId="165" formatCode="0.0%"/>
   </numFmts>
-  <fonts count="10">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -73,6 +75,16 @@
       <name val="Arial"/>
       <b val="1"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="7">
@@ -125,7 +137,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -168,6 +180,16 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -258,6 +280,26 @@
     <comment ref="I1" authorId="0" shapeId="0">
       <text>
         <t>Señales inferidas de URLs indexadas y títulos en Google. Confirmar con una visita de 30 segundos antes de escribir: año del footer, versión móvil, SSL, idiomas.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
+<file path=xl/comments/comment2.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>ThryveX</author>
+  </authors>
+  <commentList>
+    <comment ref="C1" authorId="0" shapeId="0">
+      <text>
+        <t>1 = un solo dueño, WhatsApp público, ya pagan por leads y el dolor es visible: escribir esta semana. 2 = igual de bueno pero falta un dato (dueño o número) o el ticket es menor. 3 = contactar después de tener dos casos.</t>
+      </text>
+    </comment>
+    <comment ref="G1" authorId="0" shapeId="0">
+      <text>
+        <t>Números tomados de bios de Instagram, encuentra24, Facebook y webs. Verificar en el perfil antes del primer mensaje.</t>
       </text>
     </comment>
   </commentList>
@@ -4702,7 +4744,4027 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:P61"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="4" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="6" max="6"/>
+    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="30" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
+    <col width="36" customWidth="1" min="10" max="10"/>
+    <col width="60" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
+    <col width="30" customWidth="1" min="15" max="15"/>
+    <col width="30" customWidth="1" min="16" max="16"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Nicho</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Facilidad</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Empresa / persona</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Web</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Instagram</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>WhatsApp / contacto</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Decisor</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Ya pagan por leads</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Evidencia</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Gancho (ES)</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Estado</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Fecha contacto</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Canal</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>Respuesta</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="84" customHeight="1">
+      <c r="A2" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Autos seminuevos premium</t>
+        </is>
+      </c>
+      <c r="C2" s="18" t="inlineStr">
+        <is>
+          <t>1 · Muy fácil</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>DV Motors (Costa del Este)</t>
+        </is>
+      </c>
+      <c r="E2" s="5" t="inlineStr">
+        <is>
+          <t>dvmotors.co</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>@dvmotors.pty</t>
+        </is>
+      </c>
+      <c r="G2" s="19" t="inlineStr">
+        <is>
+          <t>+507 6683-7836; sales@dvmotors.co</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>No identificado (dealer boutique, dueño presente)</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>Listados premium en encuentra24 (BMW X5, M4, Mercedes, Audi Q8); consignación y trade-in</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>29 unidades en showroom; horario L-S 9-18</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>29 carros en showroom y una sola línea de WhatsApp que cierra a las 6 pm: los leads de la noche y el domingo nadie los califica.</t>
+        </is>
+      </c>
+      <c r="L2" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M2" s="7" t="n"/>
+      <c r="N2" s="6" t="n"/>
+      <c r="O2" s="6" t="n"/>
+      <c r="P2" s="6" t="n"/>
+    </row>
+    <row r="3" ht="84" customHeight="1">
+      <c r="A3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Autos seminuevos premium</t>
+        </is>
+      </c>
+      <c r="C3" s="18" t="inlineStr">
+        <is>
+          <t>1 · Muy fácil</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>Luxury Garage Panamá + Luxury Motors Panamá (San Francisco, misma dirección)</t>
+        </is>
+      </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>luxurygaragepanama.com / luxurymotorspanama.com</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>@luxurygaragepanama (5.2K)</t>
+        </is>
+      </c>
+      <c r="G3" s="19" t="inlineStr">
+        <is>
+          <t>+507 6094-1911 / 6678-3330; tel 229-0628; info@luxurygaragepanama.com</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>No identificado (tratar ambas marcas como un solo dueño hasta confirmar)</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Perfil encuentra24 con 3 páginas de anuncios; consignación</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>Inventario Aston Martin, Ferrari, Lamborghini, Porsche; Facebook con cero reseñas; correo Gmail en una de las dos</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>Venden Ferraris y Maseratis pero su Facebook no tiene ni una reseña y la web no tiene bot: el comprador de 80 mil escribe de noche y le contestan al día siguiente.</t>
+        </is>
+      </c>
+      <c r="L3" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M3" s="7" t="n"/>
+      <c r="N3" s="6" t="n"/>
+      <c r="O3" s="6" t="n"/>
+      <c r="P3" s="6" t="n"/>
+    </row>
+    <row r="4" ht="84" customHeight="1">
+      <c r="A4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Autos seminuevos premium</t>
+        </is>
+      </c>
+      <c r="C4" s="18" t="inlineStr">
+        <is>
+          <t>1 · Muy fácil</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>UsadosPanama.com (Lumovil, Calle 50 Marbella)</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>usadospanama.com</t>
+        </is>
+      </c>
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>@usadospanama1 (24K)</t>
+        </is>
+      </c>
+      <c r="G4" s="19" t="inlineStr">
+        <is>
+          <t>WhatsApp 6426-6361; tel 214-4700; asolis@panarental.com (gerente)</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>A. Solís (gerente, ligado a Panarental)</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="inlineStr">
+        <is>
+          <t>Sección Promociones en la web; asesoría de financiamiento</t>
+        </is>
+      </c>
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>Fundada 2018; también taller</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t>Tienen promos en la web y 24K seguidores, pero el WhatsApp es un celular: los leads de las promos se pierden en el mismo chat del taller.</t>
+        </is>
+      </c>
+      <c r="L4" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M4" s="7" t="n"/>
+      <c r="N4" s="6" t="n"/>
+      <c r="O4" s="6" t="n"/>
+      <c r="P4" s="6" t="n"/>
+    </row>
+    <row r="5" ht="84" customHeight="1">
+      <c r="A5" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Autos seminuevos premium</t>
+        </is>
+      </c>
+      <c r="C5" s="18" t="inlineStr">
+        <is>
+          <t>1 · Muy fácil</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>Bottenhorn Premium Car Dealership (Costa del Este)</t>
+        </is>
+      </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>bottenhornpa.com</t>
+        </is>
+      </c>
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>@bottenhornpa; TikTok; YouTube</t>
+        </is>
+      </c>
+      <c r="G5" s="19" t="inlineStr">
+        <is>
+          <t>+507 6895-3232; info@bottenhornpa.com</t>
+        </is>
+      </c>
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>Vladimir Bottenhorn (fundador y CEO, ex BMW)</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="inlineStr">
+        <is>
+          <t>encuentra24 activo; financiamiento; 'mayor inventario de autos europeos de Panamá'</t>
+        </is>
+      </c>
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>Más de una década; negocio familiar; atiende solo por cita privada</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="inlineStr">
+        <is>
+          <t>Atienden solo por cita privada: cada mensaje de Instagram que no se responde en 10 minutos es un BMW que se va a otro showroom de Costa del Este.</t>
+        </is>
+      </c>
+      <c r="L5" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M5" s="7" t="n"/>
+      <c r="N5" s="6" t="n"/>
+      <c r="O5" s="6" t="n"/>
+      <c r="P5" s="6" t="n"/>
+    </row>
+    <row r="6" ht="84" customHeight="1">
+      <c r="A6" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Mejoras del hogar (alto ticket)</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>1 · Muy fácil</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>Cocinas y Muebles Panamá (cocinas, closets, puertas)</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>sin web / solo Instagram</t>
+        </is>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>@cocinasymueblespanama (9K)</t>
+        </is>
+      </c>
+      <c r="G6" s="19" t="inlineStr">
+        <is>
+          <t>6350-4551 (en la bio)</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="inlineStr">
+        <is>
+          <t>Bio de IG = 'cotiza al 6350-4551'; todo el embudo es Instagram a WhatsApp</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>Sin web ni Google Business fuerte</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="inlineStr">
+        <is>
+          <t>Todo el negocio vive en una bio de Instagram: sin web, y el 6350-4551 contesta solo cuando el dueño no está midiendo una cocina.</t>
+        </is>
+      </c>
+      <c r="L6" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M6" s="7" t="n"/>
+      <c r="N6" s="6" t="n"/>
+      <c r="O6" s="6" t="n"/>
+      <c r="P6" s="6" t="n"/>
+    </row>
+    <row r="7" ht="84" customHeight="1">
+      <c r="A7" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Mejoras del hogar (alto ticket)</t>
+        </is>
+      </c>
+      <c r="C7" s="18" t="inlineStr">
+        <is>
+          <t>1 · Muy fácil</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>Profil Glass (cabinas de baño, barandas, ventanas)</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>profilglasspty.com</t>
+        </is>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>@profilglasspty</t>
+        </is>
+      </c>
+      <c r="G7" s="19" t="inlineStr">
+        <is>
+          <t>+507 6430-6553; tel 391-8589</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>No identificado (Río Abajo, Plaza Gaudiano)</t>
+        </is>
+      </c>
+      <c r="I7" s="3" t="inlineStr">
+        <is>
+          <t>Web dice literalmente 'escríbenos por WhatsApp con medidas aproximadas'; horario L-S 8am-10pm</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>15+ años; portafolio en web</t>
+        </is>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>Su propia web dice 'manda las medidas por WhatsApp': un asistente que las pida, precotice y agende la visita les ahorra las 14 horas de chat diario.</t>
+        </is>
+      </c>
+      <c r="L7" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M7" s="7" t="n"/>
+      <c r="N7" s="6" t="n"/>
+      <c r="O7" s="6" t="n"/>
+      <c r="P7" s="6" t="n"/>
+    </row>
+    <row r="8" ht="84" customHeight="1">
+      <c r="A8" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Mejoras del hogar (alto ticket)</t>
+        </is>
+      </c>
+      <c r="C8" s="18" t="inlineStr">
+        <is>
+          <t>1 · Muy fácil</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>Rapid Pools / Grupo Rapid (piscinas, jacuzzis)</t>
+        </is>
+      </c>
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>rapid-pools.com / gruporapid.com</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G8" s="19" t="inlineStr">
+        <is>
+          <t>+507 6114-9653</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
+        <is>
+          <t>Gilberto Urrutia (owner, LinkedIn)</t>
+        </is>
+      </c>
+      <c r="I8" s="3" t="inlineStr">
+        <is>
+          <t>Botón 'Solicitar cotización' a WhatsApp; distribuidor Hayward; 3 sucursales (Panamá, Río Hato, David)</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>100+ clientes activos; grupo con Rapid Frío y Rapid Pest</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>Tres sucursales y tres marcas (piscinas, aire, fumigación) compartiendo un solo WhatsApp: cada lead de piscina de 20 mil compite con una queja de fumigación.</t>
+        </is>
+      </c>
+      <c r="L8" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M8" s="7" t="n"/>
+      <c r="N8" s="6" t="n"/>
+      <c r="O8" s="6" t="n"/>
+      <c r="P8" s="6" t="n"/>
+    </row>
+    <row r="9" ht="84" customHeight="1">
+      <c r="A9" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Mejoras del hogar (alto ticket)</t>
+        </is>
+      </c>
+      <c r="C9" s="18" t="inlineStr">
+        <is>
+          <t>1 · Muy fácil</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>Casabonitta Design (cocinas, closets, cuarzo)</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>casabonittadesign.com (básica)</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>@casabonittadesign (26K)</t>
+        </is>
+      </c>
+      <c r="G9" s="19" t="inlineStr">
+        <is>
+          <t>+507 6278-0450</t>
+        </is>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t>No identificado (local en Albrook Mall)</t>
+        </is>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
+          <t>26K seguidores = inversión fuerte en Instagram; local en mall 10am-8pm</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>10+ años</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>26 mil seguidores y un local en Albrook, pero cada cotización se pierde en el chat de WhatsApp mientras la web no muestra ni precios ni agenda.</t>
+        </is>
+      </c>
+      <c r="L9" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M9" s="7" t="n"/>
+      <c r="N9" s="6" t="n"/>
+      <c r="O9" s="6" t="n"/>
+      <c r="P9" s="6" t="n"/>
+    </row>
+    <row r="10" ht="84" customHeight="1">
+      <c r="A10" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Instaladores solares</t>
+        </is>
+      </c>
+      <c r="C10" s="18" t="inlineStr">
+        <is>
+          <t>1 · Muy fácil</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>Solar Power Pat S.A. (Los Pueblos)</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>solarpowerpat.net</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>FB solar.powerpat; X @SPowerPat; YouTube</t>
+        </is>
+      </c>
+      <c r="G10" s="19" t="inlineStr">
+        <is>
+          <t>6646-3171; gcomercial@solarpowerpat.com</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t>Angelo Patiño (fundador y GM desde 2014; LinkedIn)</t>
+        </is>
+      </c>
+      <c r="I10" s="3" t="inlineStr">
+        <is>
+          <t>Landings SEO por ciudad; promo financiamiento 0%; robot de limpieza SolarCleano</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>Desde 2014; Canadian Solar / Jinko</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>Publican horario L-V 8-17: el lead de Instagram que escribe viernes noche o sábado no recibe respuesta hasta el lunes.</t>
+        </is>
+      </c>
+      <c r="L10" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M10" s="7" t="n"/>
+      <c r="N10" s="6" t="n"/>
+      <c r="O10" s="6" t="n"/>
+      <c r="P10" s="6" t="n"/>
+    </row>
+    <row r="11" ht="84" customHeight="1">
+      <c r="A11" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Instaladores solares</t>
+        </is>
+      </c>
+      <c r="C11" s="18" t="inlineStr">
+        <is>
+          <t>1 · Muy fácil</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>Energiza Panamá</t>
+        </is>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>energizapanama.com</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>@energiza_panama (2.8K)</t>
+        </is>
+      </c>
+      <c r="G11" s="19" t="inlineStr">
+        <is>
+          <t>+507 6208-3614; energizapanama@gmail.com</t>
+        </is>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t>No identificado (sociedad de ~5 años)</t>
+        </is>
+      </c>
+      <c r="I11" s="3" t="inlineStr">
+        <is>
+          <t>Instagram activo; financiamiento flexible; trámites con ENSA/Naturgy como argumento</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>Desde 2018</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>Correo en Gmail y ventas por Instagram: cada DM se contesta a mano y no hay seguimiento al que pidió cotización y no cerró.</t>
+        </is>
+      </c>
+      <c r="L11" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M11" s="7" t="n"/>
+      <c r="N11" s="6" t="n"/>
+      <c r="O11" s="6" t="n"/>
+      <c r="P11" s="6" t="n"/>
+    </row>
+    <row r="12" ht="84" customHeight="1">
+      <c r="A12" s="3" t="n">
+        <v>11</v>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Instaladores solares</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>1 · Muy fácil</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>Potencia Solar (Las Mañanitas, Panamá Este)</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>potenciasolarinc.com</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G12" s="19" t="inlineStr">
+        <is>
+          <t>6440-6680; potenciasolar2025@gmail.com</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t>No identificado (empresa nueva 2025)</t>
+        </is>
+      </c>
+      <c r="I12" s="3" t="inlineStr">
+        <is>
+          <t>Proceso 'escríbenos al WhatsApp con tu factura, propuesta, visita técnica'</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>Nueva 2025; tramitan planos fotovoltaicos</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>Empresa nueva que depende 100% del WhatsApp: el flujo 'envía tu factura' es exactamente lo que un asistente IA hace 24/7 y agenda la visita.</t>
+        </is>
+      </c>
+      <c r="L12" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M12" s="7" t="n"/>
+      <c r="N12" s="6" t="n"/>
+      <c r="O12" s="6" t="n"/>
+      <c r="P12" s="6" t="n"/>
+    </row>
+    <row r="13" ht="84" customHeight="1">
+      <c r="A13" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Instaladores solares</t>
+        </is>
+      </c>
+      <c r="C13" s="18" t="inlineStr">
+        <is>
+          <t>1 · Muy fácil</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>Powerlink Solar (Av. 5 Sur y Calle 76)</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>powerlink.solar</t>
+        </is>
+      </c>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t>@powerlink.solar (1.5K)</t>
+        </is>
+      </c>
+      <c r="G13" s="19" t="inlineStr">
+        <is>
+          <t>+507 6288-8940; tel 6295-8694</t>
+        </is>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t>Camilo Amado (CEO; LinkedIn)</t>
+        </is>
+      </c>
+      <c r="I13" s="3" t="inlineStr">
+        <is>
+          <t>Mucho contenido SEO ('precio panel solar'); financiamiento propio; casos de éxito</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>30 años en ingeniería eléctrica; comercial hasta 486 paneles</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr">
+        <is>
+          <t>Invierten en SEO y financiamiento propio pero el WhatsApp es un celular: nadie califica el lead ni le pide la factura automáticamente.</t>
+        </is>
+      </c>
+      <c r="L13" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M13" s="7" t="n"/>
+      <c r="N13" s="6" t="n"/>
+      <c r="O13" s="6" t="n"/>
+      <c r="P13" s="6" t="n"/>
+    </row>
+    <row r="14" ht="84" customHeight="1">
+      <c r="A14" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Bodas y eventos</t>
+        </is>
+      </c>
+      <c r="C14" s="18" t="inlineStr">
+        <is>
+          <t>1 · Muy fácil</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>Hacienda del Alma (finca venue, Punta Barco)</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>sin web propia / ficha en ineventos.pa</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G14" s="19" t="inlineStr">
+        <is>
+          <t>6550-1269 (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>Carolyne Vergara</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>Ficha pagada en ineventos.pa; alquiler de casa completa para bodas, XV, corporativos</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>A dos minutos de Coronado</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>Una finca sin web: la novia solo sabe que existe si alguien le contesta el WhatsApp; con web y asistente, 'disponibilidad para el 14 de marzo' se responde en segundos.</t>
+        </is>
+      </c>
+      <c r="L14" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M14" s="7" t="n"/>
+      <c r="N14" s="6" t="n"/>
+      <c r="O14" s="6" t="n"/>
+      <c r="P14" s="6" t="n"/>
+    </row>
+    <row r="15" ht="84" customHeight="1">
+      <c r="A15" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Bodas y eventos</t>
+        </is>
+      </c>
+      <c r="C15" s="18" t="inlineStr">
+        <is>
+          <t>1 · Muy fácil</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Agasajos Chez Marie (catering de bodas)</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>chez-marie.com</t>
+        </is>
+      </c>
+      <c r="F15" s="3" t="inlineStr">
+        <is>
+          <t>FB @chezmariepty</t>
+        </is>
+      </c>
+      <c r="G15" s="19" t="inlineStr">
+        <is>
+          <t>WhatsApp 6200-9420; tel 269-3621 (Obarrio)</t>
+        </is>
+      </c>
+      <c r="H15" s="3" t="inlineStr">
+        <is>
+          <t>María Estela Herbruger (fundadora)</t>
+        </is>
+      </c>
+      <c r="I15" s="3" t="inlineStr">
+        <is>
+          <t>Landing 'Catering para bodas'; fichas en ineventos.com y proveedorespanama.com</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>Desde 1991 (30+ años)</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr">
+        <is>
+          <t>33 años de reputación y una web que no agenda degustaciones: cada novia pide menú por WhatsApp y espera horas la cotización.</t>
+        </is>
+      </c>
+      <c r="L15" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M15" s="7" t="n"/>
+      <c r="N15" s="6" t="n"/>
+      <c r="O15" s="6" t="n"/>
+      <c r="P15" s="6" t="n"/>
+    </row>
+    <row r="16" ht="84" customHeight="1">
+      <c r="A16" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Bodas y eventos</t>
+        </is>
+      </c>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>1 · Muy fácil</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Guedes Photographers (fotógrafos de boda)</t>
+        </is>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>guedesphotographers.com</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>@guedesphotographers</t>
+        </is>
+      </c>
+      <c r="G16" s="19" t="inlineStr">
+        <is>
+          <t>6384-0845 (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>Fabi y Miguel Guedes</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>MyWed top 3 Panamá, Wezoree; blog SEO; tarifas publicadas desde US$250/h</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>Pinterest, YouTube</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>Ya publican precio por hora: el asistente puede filtrar fecha y presupuesto y mandar el portafolio al instante mientras ellos editan.</t>
+        </is>
+      </c>
+      <c r="L16" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M16" s="7" t="n"/>
+      <c r="N16" s="6" t="n"/>
+      <c r="O16" s="6" t="n"/>
+      <c r="P16" s="6" t="n"/>
+    </row>
+    <row r="17" ht="84" customHeight="1">
+      <c r="A17" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Bodas y eventos</t>
+        </is>
+      </c>
+      <c r="C17" s="18" t="inlineStr">
+        <is>
+          <t>1 · Muy fácil</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Carlos Yap Wedding Films (videógrafo)</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>carlosyap.com</t>
+        </is>
+      </c>
+      <c r="F17" s="3" t="inlineStr">
+        <is>
+          <t>@carlosyap_ (24K)</t>
+        </is>
+      </c>
+      <c r="G17" s="19" t="inlineStr">
+        <is>
+          <t>6676-1031; info@carlosyap.com</t>
+        </is>
+      </c>
+      <c r="H17" s="3" t="inlineStr">
+        <is>
+          <t>Carlos Yap</t>
+        </is>
+      </c>
+      <c r="I17" s="3" t="inlineStr">
+        <is>
+          <t>Wezoree Top 5 Panamá, Top 100 global</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>10+ años; 90+ bodas</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
+          <t>Cuando Carlos está grabando una boda no puede contestar; justo ese sábado es cuando más parejas comprometidas escriben.</t>
+        </is>
+      </c>
+      <c r="L17" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M17" s="7" t="n"/>
+      <c r="N17" s="6" t="n"/>
+      <c r="O17" s="6" t="n"/>
+      <c r="P17" s="6" t="n"/>
+    </row>
+    <row r="18" ht="84" customHeight="1">
+      <c r="A18" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Agentes y alquiler corto</t>
+        </is>
+      </c>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>1 · Muy fácil</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Rentyfive (Marcela Macías) · administradora</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>rentyfive.com + linktr.ee/marcelamacias_rentyfive</t>
+        </is>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>@marcelamacias_rentyfive</t>
+        </is>
+      </c>
+      <c r="G18" s="19" t="inlineStr">
+        <is>
+          <t>+507 6877-0777 / 6723-4323; info@myrentyfive.com</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>Marcela Macías (fundadora, marca personal)</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>Linktree, IG personal, web bilingüe</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>25+ propiedades; Superhost 4.9; desde 2018</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>Con 25 propiedades, cada consulta de 'disponibilidad y precio' que llega de noche por WhatsApp es una reserva que se va a Booking.</t>
+        </is>
+      </c>
+      <c r="L18" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M18" s="7" t="n"/>
+      <c r="N18" s="6" t="n"/>
+      <c r="O18" s="6" t="n"/>
+      <c r="P18" s="6" t="n"/>
+    </row>
+    <row r="19" ht="84" customHeight="1">
+      <c r="A19" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Agentes y alquiler corto</t>
+        </is>
+      </c>
+      <c r="C19" s="18" t="inlineStr">
+        <is>
+          <t>1 · Muy fácil</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Aldo Stagnaro · agente</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>aldostagnaro.com</t>
+        </is>
+      </c>
+      <c r="F19" s="3" t="inlineStr">
+        <is>
+          <t>@aldostagnaro</t>
+        </is>
+      </c>
+      <c r="G19" s="19" t="inlineStr">
+        <is>
+          <t>+507 6674-8054 (WA); oficina 223-6899</t>
+        </is>
+      </c>
+      <c r="H19" s="3" t="inlineStr">
+        <is>
+          <t>Aldo Stagnaro (oficina propia con su esposa Cristina; ex presidente de ACOBIR)</t>
+        </is>
+      </c>
+      <c r="I19" s="3" t="inlineStr">
+        <is>
+          <t>Podcast 'Compradores Inmobiliarios' (4 temporadas), YouTube, TikTok, MLS ACOBIR</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>22-27 años; citado en La Prensa</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>Usted produce podcast, YouTube y TikTok, pero cada oyente que escribe de noche cae en el mismo WhatsApp de tres personas que están en showings.</t>
+        </is>
+      </c>
+      <c r="L19" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M19" s="7" t="n"/>
+      <c r="N19" s="6" t="n"/>
+      <c r="O19" s="6" t="n"/>
+      <c r="P19" s="6" t="n"/>
+    </row>
+    <row r="20" ht="84" customHeight="1">
+      <c r="A20" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Agentes y alquiler corto</t>
+        </is>
+      </c>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>1 · Muy fácil</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>DM Real Estate Panamá · agente independiente</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>sin web / solo IG + Threads + YouTube</t>
+        </is>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>@dmrealestatepanama (14K) + @dmluxuryrealestatepty</t>
+        </is>
+      </c>
+      <c r="G20" s="19" t="inlineStr">
+        <is>
+          <t>+507 6244-0638 (wa.me)</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>No visible (12 años de experiencia)</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>Perfil pago de agente en encuentra24; dos cuentas IG; YouTube</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>12 años</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t>14 mil seguidores y cero web: cada lead de reel termina en un DM manual que nadie califica por presupuesto ni zona.</t>
+        </is>
+      </c>
+      <c r="L20" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M20" s="7" t="n"/>
+      <c r="N20" s="6" t="n"/>
+      <c r="O20" s="6" t="n"/>
+      <c r="P20" s="6" t="n"/>
+    </row>
+    <row r="21" ht="84" customHeight="1">
+      <c r="A21" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Agentes y alquiler corto</t>
+        </is>
+      </c>
+      <c r="C21" s="18" t="inlineStr">
+        <is>
+          <t>1 · Muy fácil</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Panama Sarah / Panama Holiday Homes (Coronado) · administradora</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>panamasarah.com</t>
+        </is>
+      </c>
+      <c r="F21" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G21" s="19" t="inlineStr">
+        <is>
+          <t>+507 6671-1444 (WA)</t>
+        </is>
+      </c>
+      <c r="H21" s="3" t="inlineStr">
+        <is>
+          <t>Sarah</t>
+        </is>
+      </c>
+      <c r="I21" s="3" t="inlineStr">
+        <is>
+          <t>Airbnb, VRBO, TripAdvisor</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>Superhost; VRBO Premier Host; TripAdvisor Certificate of Excellence; 18 años en Panamá</t>
+        </is>
+      </c>
+      <c r="K21" s="3" t="inlineStr">
+        <is>
+          <t>Superhost en tres plataformas, pero su web no reserva directo ni responde sola: paga 15% de comisión por huéspedes que ya la buscan por nombre.</t>
+        </is>
+      </c>
+      <c r="L21" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M21" s="7" t="n"/>
+      <c r="N21" s="6" t="n"/>
+      <c r="O21" s="6" t="n"/>
+      <c r="P21" s="6" t="n"/>
+    </row>
+    <row r="22" ht="84" customHeight="1">
+      <c r="A22" s="3" t="n">
+        <v>21</v>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Autos seminuevos premium</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>2 · Fácil</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Super Autos Panamá (Vía España / Vía Porras)</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>superautospanama.com</t>
+        </is>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>@superautospty (69K); TikTok 11K</t>
+        </is>
+      </c>
+      <c r="G22" s="19" t="inlineStr">
+        <is>
+          <t>WhatsApp 6013-2000 / 6023-3708 / 6015-5554; Publicidad@superautospty.net</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>Correo 'Publicidad@' = presupuesto de pauta; 6 páginas en encuentra24; TikTok activo</t>
+        </is>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>Dos sucursales; inventario amplio</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>69K seguidores y tres números de WhatsApp distintos: nadie sabe cuál lead ya se atendió ni quién hizo seguimiento.</t>
+        </is>
+      </c>
+      <c r="L22" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M22" s="7" t="n"/>
+      <c r="N22" s="6" t="n"/>
+      <c r="O22" s="6" t="n"/>
+      <c r="P22" s="6" t="n"/>
+    </row>
+    <row r="23" ht="84" customHeight="1">
+      <c r="A23" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Autos seminuevos premium</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>2 · Fácil</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Full Cars Panamá (Vía Israel / San Francisco)</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>fullcarspanama.com</t>
+        </is>
+      </c>
+      <c r="F23" s="3" t="inlineStr">
+        <is>
+          <t>Facebook 13K; IG @_fullcars__</t>
+        </is>
+      </c>
+      <c r="G23" s="19" t="inlineStr">
+        <is>
+          <t>+507 6671-2525; ventas@fullcarspanama.com</t>
+        </is>
+      </c>
+      <c r="H23" s="3" t="inlineStr">
+        <is>
+          <t>Claudio Downs (presidente, desde 2009)</t>
+        </is>
+      </c>
+      <c r="I23" s="3" t="inlineStr">
+        <is>
+          <t>Web con calculadora de avalúo y páginas SEO por marca; encuentra24</t>
+        </is>
+      </c>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>Facebook 96% recomendado (17 reseñas); dos sucursales; garantía 6 meses</t>
+        </is>
+      </c>
+      <c r="K23" s="3" t="inlineStr">
+        <is>
+          <t>Invierten en SEO y calculadora de avalúo, pero el que llena el formulario a las 9 pm recibe respuesta humana al otro día.</t>
+        </is>
+      </c>
+      <c r="L23" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M23" s="7" t="n"/>
+      <c r="N23" s="6" t="n"/>
+      <c r="O23" s="6" t="n"/>
+      <c r="P23" s="6" t="n"/>
+    </row>
+    <row r="24" ht="84" customHeight="1">
+      <c r="A24" s="3" t="n">
+        <v>23</v>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Autos seminuevos premium</t>
+        </is>
+      </c>
+      <c r="C24" s="6" t="inlineStr">
+        <is>
+          <t>2 · Fácil</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Autos Usados Panamá (Juan Díaz / Brisas)</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>autosusadospanama.com</t>
+        </is>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>@autosusadospa (52K); Threads</t>
+        </is>
+      </c>
+      <c r="G24" s="19" t="inlineStr">
+        <is>
+          <t>WhatsApp 6509-9864 / 6669-5101; ventas@autosusadospanama.com</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>'Financiamiento disponible' en bio; trade-in</t>
+        </is>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>Horario L-V 9-5, sáb 9-4</t>
+        </is>
+      </c>
+      <c r="K24" s="3" t="inlineStr">
+        <is>
+          <t>52K seguidores en Instagram y cierran a las 5 pm: dos tercios de los mensajes llegan cuando no hay nadie.</t>
+        </is>
+      </c>
+      <c r="L24" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M24" s="7" t="n"/>
+      <c r="N24" s="6" t="n"/>
+      <c r="O24" s="6" t="n"/>
+      <c r="P24" s="6" t="n"/>
+    </row>
+    <row r="25" ht="84" customHeight="1">
+      <c r="A25" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Autos seminuevos premium</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>2 · Fácil</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Carspot Panamá (Tumba Muerto + Cincuentenario + Chiriquí)</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>carspotpanama.com</t>
+        </is>
+      </c>
+      <c r="F25" s="3" t="inlineStr">
+        <is>
+          <t>@carspotpanama</t>
+        </is>
+      </c>
+      <c r="G25" s="19" t="inlineStr">
+        <is>
+          <t>WhatsApp 6894-4194 / 6896-2851; chat 6642-8284; tel 236-0091; info@carspotpanama.com</t>
+        </is>
+      </c>
+      <c r="H25" s="3" t="inlineStr">
+        <is>
+          <t>Moisés R. Novoa (usuario encuentra24 con 11 páginas de anuncios)</t>
+        </is>
+      </c>
+      <c r="I25" s="3" t="inlineStr">
+        <is>
+          <t>11 páginas en encuentra24 (paquete premium); financiamiento</t>
+        </is>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>15-21 años; tres sucursales</t>
+        </is>
+      </c>
+      <c r="K25" s="3" t="inlineStr">
+        <is>
+          <t>Pagan paquete grande en encuentra24 y reparten los leads entre cuatro celulares: nadie mide cuántos se convierten.</t>
+        </is>
+      </c>
+      <c r="L25" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M25" s="7" t="n"/>
+      <c r="N25" s="6" t="n"/>
+      <c r="O25" s="6" t="n"/>
+      <c r="P25" s="6" t="n"/>
+    </row>
+    <row r="26" ht="84" customHeight="1">
+      <c r="A26" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Autos seminuevos premium</t>
+        </is>
+      </c>
+      <c r="C26" s="6" t="inlineStr">
+        <is>
+          <t>2 · Fácil</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Champion Motors (Transístmica)</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>championmotors.com.pa</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>@championmotorspanama (110K)</t>
+        </is>
+      </c>
+      <c r="G26" s="19" t="inlineStr">
+        <is>
+          <t>WhatsApp +507 6673-4508; tel 260-1461</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>Financiamiento 'aprobación en 24 h'; inspección 100+ puntos; encuentra24</t>
+        </is>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>Google 4.8 (127 reseñas); 23 años</t>
+        </is>
+      </c>
+      <c r="K26" s="3" t="inlineStr">
+        <is>
+          <t>110K seguidores y prometen aprobación en 24 horas: el bot puede precalificar el crédito en dos minutos antes de que el vendedor levante el teléfono.</t>
+        </is>
+      </c>
+      <c r="L26" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M26" s="7" t="n"/>
+      <c r="N26" s="6" t="n"/>
+      <c r="O26" s="6" t="n"/>
+      <c r="P26" s="6" t="n"/>
+    </row>
+    <row r="27" ht="84" customHeight="1">
+      <c r="A27" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Mejoras del hogar (alto ticket)</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>2 · Fácil</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Arte Cocinas S.A.</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>artecocinas.net + landing cocinas.artecocinas.net</t>
+        </is>
+      </c>
+      <c r="F27" s="3" t="inlineStr">
+        <is>
+          <t>@artecocinas.s.a (4.7K)</t>
+        </is>
+      </c>
+      <c r="G27" s="19" t="inlineStr">
+        <is>
+          <t>+507 6568-1896; tel 396-5663; ventas@artecocinas.net</t>
+        </is>
+      </c>
+      <c r="H27" s="3" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="I27" s="3" t="inlineStr">
+        <is>
+          <t>Landing separada (típico de campañas de Ads); ficha pagada en Construex</t>
+        </is>
+      </c>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>15+ años</t>
+        </is>
+      </c>
+      <c r="K27" s="3" t="inlineStr">
+        <is>
+          <t>Pagan una landing para captar leads de cocinas y luego los mandan a un WhatsApp sin seguimiento ni recordatorio de visita.</t>
+        </is>
+      </c>
+      <c r="L27" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M27" s="7" t="n"/>
+      <c r="N27" s="6" t="n"/>
+      <c r="O27" s="6" t="n"/>
+      <c r="P27" s="6" t="n"/>
+    </row>
+    <row r="28" ht="84" customHeight="1">
+      <c r="A28" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Mejoras del hogar (alto ticket)</t>
+        </is>
+      </c>
+      <c r="C28" s="6" t="inlineStr">
+        <is>
+          <t>2 · Fácil</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Maobe Muebles (cocinas modulares, closets)</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>maobemuebles.com (blog SEO activo)</t>
+        </is>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>@maobemueblespanama</t>
+        </is>
+      </c>
+      <c r="G28" s="19" t="inlineStr">
+        <is>
+          <t>+507 6938-4466; tel 318-1238</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>No identificado (Brisas del Golf)</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>Blog SEO + ficha Construex + 'consulta online y visita a domicilio'</t>
+        </is>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>Proyectos residenciales y oficinas</t>
+        </is>
+      </c>
+      <c r="K28" s="3" t="inlineStr">
+        <is>
+          <t>Invierten en blog y SEO, pero el lead que llega a las 9 pm por WhatsApp espera hasta el día siguiente para saber si pueden medir.</t>
+        </is>
+      </c>
+      <c r="L28" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M28" s="7" t="n"/>
+      <c r="N28" s="6" t="n"/>
+      <c r="O28" s="6" t="n"/>
+      <c r="P28" s="6" t="n"/>
+    </row>
+    <row r="29" ht="84" customHeight="1">
+      <c r="A29" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="B29" s="3" t="inlineStr">
+        <is>
+          <t>Mejoras del hogar (alto ticket)</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
+        <is>
+          <t>2 · Fácil</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>Ventanas Vigil / Crialvi (aluminio y vidrio templado)</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>ventanasvigil.com</t>
+        </is>
+      </c>
+      <c r="F29" s="3" t="inlineStr">
+        <is>
+          <t>FB ventanasvigil</t>
+        </is>
+      </c>
+      <c r="G29" s="19" t="inlineStr">
+        <is>
+          <t>+507 6017-7949; tel 258-1599; ventascrialvi.sa@gmail.com</t>
+        </is>
+      </c>
+      <c r="H29" s="3" t="inlineStr">
+        <is>
+          <t>Familia Vigil</t>
+        </is>
+      </c>
+      <c r="I29" s="3" t="inlineStr">
+        <is>
+          <t>'Cotiza por WhatsApp' en web y Facebook; cobertura Panamá + La Chorrera</t>
+        </is>
+      </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>14-15 años; fábrica propia</t>
+        </is>
+      </c>
+      <c r="K29" s="3" t="inlineStr">
+        <is>
+          <t>Fábrica con 15 años y dos zonas de cobertura, pero el cliente aún tiene que mandar medidas por WhatsApp y esperar a que alguien del taller responda.</t>
+        </is>
+      </c>
+      <c r="L29" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M29" s="7" t="n"/>
+      <c r="N29" s="6" t="n"/>
+      <c r="O29" s="6" t="n"/>
+      <c r="P29" s="6" t="n"/>
+    </row>
+    <row r="30" ht="84" customHeight="1">
+      <c r="A30" s="3" t="n">
+        <v>29</v>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Mejoras del hogar (alto ticket)</t>
+        </is>
+      </c>
+      <c r="C30" s="6" t="inlineStr">
+        <is>
+          <t>2 · Fácil</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>The Glass House Panamá (puertas de baño templadas, barandas)</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>theglasshousepanama.com (tienda online)</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>TikTok @theglasshousepanama</t>
+        </is>
+      </c>
+      <c r="G30" s="19" t="inlineStr">
+        <is>
+          <t>6002-4099; contacto@theglasshousepanama.com</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>No identificado (Parque Lefevre)</t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>TikTok con hashtags de Costa del Este y Paitilla; tienda online</t>
+        </is>
+      </c>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="K30" s="3" t="inlineStr">
+        <is>
+          <t>Hacen videos en TikTok para Paitilla y Costa del Este, pero la cotización de una puerta de baño sigue dependiendo de que alguien lea el WhatsApp.</t>
+        </is>
+      </c>
+      <c r="L30" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M30" s="7" t="n"/>
+      <c r="N30" s="6" t="n"/>
+      <c r="O30" s="6" t="n"/>
+      <c r="P30" s="6" t="n"/>
+    </row>
+    <row r="31" ht="84" customHeight="1">
+      <c r="A31" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t>Mejoras del hogar (alto ticket)</t>
+        </is>
+      </c>
+      <c r="C31" s="6" t="inlineStr">
+        <is>
+          <t>2 · Fácil</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>Remodela Panamá (Proyectos Castañedas)</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>remodelapanama.com + remodelapma.com</t>
+        </is>
+      </c>
+      <c r="F31" s="3" t="inlineStr">
+        <is>
+          <t>@remodelapanama</t>
+        </is>
+      </c>
+      <c r="G31" s="19" t="inlineStr">
+        <is>
+          <t>+507 6724-5390</t>
+        </is>
+      </c>
+      <c r="H31" s="3" t="inlineStr">
+        <is>
+          <t>Familia Castañeda</t>
+        </is>
+      </c>
+      <c r="I31" s="3" t="inlineStr">
+        <is>
+          <t>Dos dominios + blog de precios 2025; 'cotiza por WhatsApp e Instagram'</t>
+        </is>
+      </c>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>20+ años</t>
+        </is>
+      </c>
+      <c r="K31" s="3" t="inlineStr">
+        <is>
+          <t>Escriben blogs de '¿cuánto cuesta remodelar?' para atraer tráfico y luego el visitante termina en un WhatsApp que no califica ni agenda la visita técnica.</t>
+        </is>
+      </c>
+      <c r="L31" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M31" s="7" t="n"/>
+      <c r="N31" s="6" t="n"/>
+      <c r="O31" s="6" t="n"/>
+      <c r="P31" s="6" t="n"/>
+    </row>
+    <row r="32" ht="84" customHeight="1">
+      <c r="A32" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Mejoras del hogar (alto ticket)</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>2 · Fácil</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>Renovation PA (remodelación llave en mano, Airbnb, playa)</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>renovationpa.com</t>
+        </is>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>@renovationpa</t>
+        </is>
+      </c>
+      <c r="G32" s="19" t="inlineStr">
+        <is>
+          <t>+507 6584-7309</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>No identificado (Bal Harbour)</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>'Consulta gratis por WhatsApp'; portafolio Coronado, Multimax</t>
+        </is>
+      </c>
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>Proyectos en Panamá, Coronado y Miami</t>
+        </is>
+      </c>
+      <c r="K32" s="3" t="inlineStr">
+        <is>
+          <t>Venden remodelaciones llave en mano a dueños de Airbnb que escriben de noche y fin de semana, justo cuando nadie contesta.</t>
+        </is>
+      </c>
+      <c r="L32" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M32" s="7" t="n"/>
+      <c r="N32" s="6" t="n"/>
+      <c r="O32" s="6" t="n"/>
+      <c r="P32" s="6" t="n"/>
+    </row>
+    <row r="33" ht="84" customHeight="1">
+      <c r="A33" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="B33" s="3" t="inlineStr">
+        <is>
+          <t>Mejoras del hogar (alto ticket)</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>2 · Fácil</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>DiraSmart (domótica KNX)</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>dirasmart.com</t>
+        </is>
+      </c>
+      <c r="F33" s="3" t="inlineStr">
+        <is>
+          <t>@dirasmart</t>
+        </is>
+      </c>
+      <c r="G33" s="19" t="inlineStr">
+        <is>
+          <t>+507 6595-6439</t>
+        </is>
+      </c>
+      <c r="H33" s="3" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="I33" s="3" t="inlineStr">
+        <is>
+          <t>Página de ofertas y de reseñas; KNX Partner</t>
+        </is>
+      </c>
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>Proyectos residenciales y hoteles</t>
+        </is>
+      </c>
+      <c r="K33" s="3" t="inlineStr">
+        <is>
+          <t>Prometen 'soporte directo por WhatsApp con quien instaló': con dos o tres técnicos eso no escala; un asistente que filtre soporte de venta nueva les devuelve horas.</t>
+        </is>
+      </c>
+      <c r="L33" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M33" s="7" t="n"/>
+      <c r="N33" s="6" t="n"/>
+      <c r="O33" s="6" t="n"/>
+      <c r="P33" s="6" t="n"/>
+    </row>
+    <row r="34" ht="84" customHeight="1">
+      <c r="A34" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Instaladores solares</t>
+        </is>
+      </c>
+      <c r="C34" s="6" t="inlineStr">
+        <is>
+          <t>2 · Fácil</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>Bahía Solar Energy</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>bahiasolarenergy.com</t>
+        </is>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>@bahiasolarenergy</t>
+        </is>
+      </c>
+      <c r="G34" s="19" t="inlineStr">
+        <is>
+          <t>+507 6796-0238; ventas@bahiasolarenergy.com</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>Página SEO 'Precio de paneles solares en Panamá 2026'; Cámara Solar; testimonios</t>
+        </is>
+      </c>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>Equipo con hasta 15 años</t>
+        </is>
+      </c>
+      <c r="K34" s="3" t="inlineStr">
+        <is>
+          <t>Captan tráfico con la página de precios 2026 pero el visitante termina en un WhatsApp humano; el que pide precio a las 9 pm espera al día siguiente.</t>
+        </is>
+      </c>
+      <c r="L34" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M34" s="7" t="n"/>
+      <c r="N34" s="6" t="n"/>
+      <c r="O34" s="6" t="n"/>
+      <c r="P34" s="6" t="n"/>
+    </row>
+    <row r="35" ht="84" customHeight="1">
+      <c r="A35" s="3" t="n">
+        <v>34</v>
+      </c>
+      <c r="B35" s="3" t="inlineStr">
+        <is>
+          <t>Instaladores solares</t>
+        </is>
+      </c>
+      <c r="C35" s="6" t="inlineStr">
+        <is>
+          <t>2 · Fácil</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>Paneles Solares en Panamá</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>panelessolaresenpanama.com</t>
+        </is>
+      </c>
+      <c r="F35" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G35" s="19" t="inlineStr">
+        <is>
+          <t>+507 6944-1778</t>
+        </is>
+      </c>
+      <c r="H35" s="3" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="I35" s="3" t="inlineStr">
+        <is>
+          <t>Dominio exact-match para SEO/Ads; promesa 'respondemos en pocas horas'</t>
+        </is>
+      </c>
+      <c r="J35" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="K35" s="3" t="inlineStr">
+        <is>
+          <t>Prometen responder 'en pocas horas': con un asistente la respuesta es en segundos y el lead no se enfría.</t>
+        </is>
+      </c>
+      <c r="L35" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M35" s="7" t="n"/>
+      <c r="N35" s="6" t="n"/>
+      <c r="O35" s="6" t="n"/>
+      <c r="P35" s="6" t="n"/>
+    </row>
+    <row r="36" ht="84" customHeight="1">
+      <c r="A36" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Instaladores solares</t>
+        </is>
+      </c>
+      <c r="C36" s="6" t="inlineStr">
+        <is>
+          <t>2 · Fácil</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>Solar Panel Panama (expats)</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>solarpanelpanama.com</t>
+        </is>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G36" s="19" t="inlineStr">
+        <is>
+          <t>6565-4145; info@solarpanelpanama.com</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>Web bilingüe orientada a búsqueda en inglés</t>
+        </is>
+      </c>
+      <c r="J36" s="3" t="inlineStr">
+        <is>
+          <t>Horario L-V 8-17</t>
+        </is>
+      </c>
+      <c r="K36" s="3" t="inlineStr">
+        <is>
+          <t>Atienden expats pero solo de lunes a viernes de 8 a 5: el extranjero que escribe en inglés un domingo no recibe respuesta.</t>
+        </is>
+      </c>
+      <c r="L36" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M36" s="7" t="n"/>
+      <c r="N36" s="6" t="n"/>
+      <c r="O36" s="6" t="n"/>
+      <c r="P36" s="6" t="n"/>
+    </row>
+    <row r="37" ht="84" customHeight="1">
+      <c r="A37" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="B37" s="3" t="inlineStr">
+        <is>
+          <t>Instaladores solares</t>
+        </is>
+      </c>
+      <c r="C37" s="6" t="inlineStr">
+        <is>
+          <t>2 · Fácil</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>Panama Solar Solutions (Carrasquilla)</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr">
+        <is>
+          <t>panamasolarsolutions.com</t>
+        </is>
+      </c>
+      <c r="F37" s="3" t="inlineStr">
+        <is>
+          <t>FB e IG</t>
+        </is>
+      </c>
+      <c r="G37" s="19" t="inlineStr">
+        <is>
+          <t>6230-3333</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="I37" s="3" t="inlineStr">
+        <is>
+          <t>Asesoría de cálculo de costos y ROI</t>
+        </is>
+      </c>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="K37" s="3" t="inlineStr">
+        <is>
+          <t>Web sencilla sin cotizador: el cliente tiene que llamar o escribir y esperar a que un técnico le calcule el sistema.</t>
+        </is>
+      </c>
+      <c r="L37" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M37" s="7" t="n"/>
+      <c r="N37" s="6" t="n"/>
+      <c r="O37" s="6" t="n"/>
+      <c r="P37" s="6" t="n"/>
+    </row>
+    <row r="38" ht="84" customHeight="1">
+      <c r="A38" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Instaladores solares</t>
+        </is>
+      </c>
+      <c r="C38" s="6" t="inlineStr">
+        <is>
+          <t>2 · Fácil</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>SiempreSol Panamá (Boquete, expats)</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>siempresolpanama.com</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>FB siempresolpanama (1 reseña)</t>
+        </is>
+      </c>
+      <c r="G38" s="19" t="inlineStr">
+        <is>
+          <t>+507 6631-9193; alain@siempresolpanama.com</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>Alain (fundador aparente)</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="inlineStr">
+        <is>
+          <t>Listado en igopanama.com; web en inglés</t>
+        </is>
+      </c>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>Desde 2018; hasta 150+ paneles</t>
+        </is>
+      </c>
+      <c r="K38" s="3" t="inlineStr">
+        <is>
+          <t>Mercado expat en Boquete con una reseña en Facebook y respuesta manual en inglés: pierden referidos y no piden reseñas después de instalar.</t>
+        </is>
+      </c>
+      <c r="L38" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M38" s="7" t="n"/>
+      <c r="N38" s="6" t="n"/>
+      <c r="O38" s="6" t="n"/>
+      <c r="P38" s="6" t="n"/>
+    </row>
+    <row r="39" ht="84" customHeight="1">
+      <c r="A39" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="B39" s="3" t="inlineStr">
+        <is>
+          <t>Instaladores solares</t>
+        </is>
+      </c>
+      <c r="C39" s="6" t="inlineStr">
+        <is>
+          <t>2 · Fácil</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>Electrysol S.A. (David, Chiriquí)</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>electrysol.com</t>
+        </is>
+      </c>
+      <c r="F39" s="3" t="inlineStr">
+        <is>
+          <t>@electrysolpanama</t>
+        </is>
+      </c>
+      <c r="G39" s="19" t="inlineStr">
+        <is>
+          <t>774-1080 / 6258-7635 (WhatsApp)</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="inlineStr">
+        <is>
+          <t>Víctor Saldaña (rol por confirmar)</t>
+        </is>
+      </c>
+      <c r="I39" s="3" t="inlineStr">
+        <is>
+          <t>Infoguía, WhatsApp e IG; 'primera empresa solar del país'</t>
+        </is>
+      </c>
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>Desde 1992; garantías 26+ años</t>
+        </is>
+      </c>
+      <c r="K39" s="3" t="inlineStr">
+        <is>
+          <t>33 años instalando y una web vieja: la reputación no se ve en Google ni en Instagram, y el WhatsApp sigue siendo un celular de oficina.</t>
+        </is>
+      </c>
+      <c r="L39" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M39" s="7" t="n"/>
+      <c r="N39" s="6" t="n"/>
+      <c r="O39" s="6" t="n"/>
+      <c r="P39" s="6" t="n"/>
+    </row>
+    <row r="40" ht="84" customHeight="1">
+      <c r="A40" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Bodas y eventos</t>
+        </is>
+      </c>
+      <c r="C40" s="6" t="inlineStr">
+        <is>
+          <t>2 · Fácil</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>Paola Mantilla Events (wedding planner)</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>paolamantilla.com (Squarespace)</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G40" s="19" t="inlineStr">
+        <is>
+          <t>6675-4685; info@paolamantilla.com (Punta Paitilla, L-V 9-7)</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>Paola Mantilla</t>
+        </is>
+      </c>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>Wezoree con 3 premios, Top 5 Panamá</t>
+        </is>
+      </c>
+      <c r="J40" s="3" t="inlineStr">
+        <is>
+          <t>Desde 2007</t>
+        </is>
+      </c>
+      <c r="K40" s="3" t="inlineStr">
+        <is>
+          <t>Oficina de lunes a viernes de 9 a 7: las parejas escriben sábado y domingo. Un asistente que responda y agende el lunes a primera hora cierra ese hueco.</t>
+        </is>
+      </c>
+      <c r="L40" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M40" s="7" t="n"/>
+      <c r="N40" s="6" t="n"/>
+      <c r="O40" s="6" t="n"/>
+      <c r="P40" s="6" t="n"/>
+    </row>
+    <row r="41" ht="84" customHeight="1">
+      <c r="A41" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="B41" s="3" t="inlineStr">
+        <is>
+          <t>Bodas y eventos</t>
+        </is>
+      </c>
+      <c r="C41" s="6" t="inlineStr">
+        <is>
+          <t>2 · Fácil</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>MCH The Bride Atelier (planner, decor, floristería)</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>mchthebrideatelier.com</t>
+        </is>
+      </c>
+      <c r="F41" s="3" t="inlineStr">
+        <is>
+          <t>vía web</t>
+        </is>
+      </c>
+      <c r="G41" s="19" t="inlineStr">
+        <is>
+          <t>6998-5134; info@mchthebrideatelier.com (Condado del Rey)</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="inlineStr">
+        <is>
+          <t>No identificado (certificada ABC)</t>
+        </is>
+      </c>
+      <c r="I41" s="3" t="inlineStr">
+        <is>
+          <t>Ya ofrece 'reserva en línea o por WhatsApp'; en Asoflor</t>
+        </is>
+      </c>
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>20+ años</t>
+        </is>
+      </c>
+      <c r="K41" s="3" t="inlineStr">
+        <is>
+          <t>Ya invita a reservar por WhatsApp; falta que ese WhatsApp califique y agende solo, en vez de ser otro chat pendiente.</t>
+        </is>
+      </c>
+      <c r="L41" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M41" s="7" t="n"/>
+      <c r="N41" s="6" t="n"/>
+      <c r="O41" s="6" t="n"/>
+      <c r="P41" s="6" t="n"/>
+    </row>
+    <row r="42" ht="84" customHeight="1">
+      <c r="A42" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Bodas y eventos</t>
+        </is>
+      </c>
+      <c r="C42" s="6" t="inlineStr">
+        <is>
+          <t>2 · Fácil</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>Bacioni Eventos (wedding planners)</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>bacionieventos.com</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>FB + IG</t>
+        </is>
+      </c>
+      <c r="G42" s="19" t="inlineStr">
+        <is>
+          <t>6065-8644; info@bacionieventos.com</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
+        <is>
+          <t>Alyssa Madrid</t>
+        </is>
+      </c>
+      <c r="I42" s="3" t="inlineStr">
+        <is>
+          <t>Listada en ineventos.com</t>
+        </is>
+      </c>
+      <c r="J42" s="3" t="inlineStr">
+        <is>
+          <t>Certificada 2017 (~8 años)</t>
+        </is>
+      </c>
+      <c r="K42" s="3" t="inlineStr">
+        <is>
+          <t>Equipo pequeño que vive del DM: cada cotización se escribe a mano y la mitad de las consultas nunca recibe seguimiento.</t>
+        </is>
+      </c>
+      <c r="L42" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M42" s="7" t="n"/>
+      <c r="N42" s="6" t="n"/>
+      <c r="O42" s="6" t="n"/>
+      <c r="P42" s="6" t="n"/>
+    </row>
+    <row r="43" ht="84" customHeight="1">
+      <c r="A43" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="B43" s="3" t="inlineStr">
+        <is>
+          <t>Bodas y eventos</t>
+        </is>
+      </c>
+      <c r="C43" s="6" t="inlineStr">
+        <is>
+          <t>2 · Fácil</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>Casa Greca (venue frente al mar, Playa Blanca)</t>
+        </is>
+      </c>
+      <c r="E43" s="5" t="inlineStr">
+        <is>
+          <t>casagrecapa.com</t>
+        </is>
+      </c>
+      <c r="F43" s="3" t="inlineStr">
+        <is>
+          <t>@casagrecapa</t>
+        </is>
+      </c>
+      <c r="G43" s="19" t="inlineStr">
+        <is>
+          <t>6221-2892; casagrecapa@gmail.com</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="inlineStr">
+        <is>
+          <t>Familia propietaria</t>
+        </is>
+      </c>
+      <c r="I43" s="3" t="inlineStr">
+        <is>
+          <t>Booking, TripAdvisor, Airbnb (comisiones); Instagram activo</t>
+        </is>
+      </c>
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t>Reseñas en TripAdvisor/Booking</t>
+        </is>
+      </c>
+      <c r="K43" s="3" t="inlineStr">
+        <is>
+          <t>Paga comisión a Booking y Airbnb por noches, pero las bodas (el ticket de 10 a 30 mil) llegan por DM y se pierden entre consultas de day pass.</t>
+        </is>
+      </c>
+      <c r="L43" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M43" s="7" t="n"/>
+      <c r="N43" s="6" t="n"/>
+      <c r="O43" s="6" t="n"/>
+      <c r="P43" s="6" t="n"/>
+    </row>
+    <row r="44" ht="84" customHeight="1">
+      <c r="A44" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Bodas y eventos</t>
+        </is>
+      </c>
+      <c r="C44" s="6" t="inlineStr">
+        <is>
+          <t>2 · Fácil</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>Hacienda Los Molinos (venue en Boquete, hasta 250 pax)</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>losmolinoshotel.com</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>@haciendalosmolinosboquete (6K)</t>
+        </is>
+      </c>
+      <c r="G44" s="19" t="inlineStr">
+        <is>
+          <t>6676-0653; 730-8313; reservas@losmolinoshotel.com</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
+        <is>
+          <t>Hotel boutique independiente</t>
+        </is>
+      </c>
+      <c r="I44" s="3" t="inlineStr">
+        <is>
+          <t>Ficha en ineventos.pa; páginas SEO 'lugares para bodas en Boquete'</t>
+        </is>
+      </c>
+      <c r="J44" s="3" t="inlineStr">
+        <is>
+          <t>6 habitaciones + 10 villas; menús de boda publicados</t>
+        </is>
+      </c>
+      <c r="K44" s="3" t="inlineStr">
+        <is>
+          <t>Bodas destino desde la ciudad y el extranjero escriben en husos horarios distintos; el que responde de madrugada se queda con el tour por la finca.</t>
+        </is>
+      </c>
+      <c r="L44" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M44" s="7" t="n"/>
+      <c r="N44" s="6" t="n"/>
+      <c r="O44" s="6" t="n"/>
+      <c r="P44" s="6" t="n"/>
+    </row>
+    <row r="45" ht="84" customHeight="1">
+      <c r="A45" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="B45" s="3" t="inlineStr">
+        <is>
+          <t>Bodas y eventos</t>
+        </is>
+      </c>
+      <c r="C45" s="6" t="inlineStr">
+        <is>
+          <t>2 · Fácil</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>Le Fleur by Michelle Vallarino (floral + decoración de bodas)</t>
+        </is>
+      </c>
+      <c r="E45" s="5" t="inlineStr">
+        <is>
+          <t>lefleurbymichellevallarino.com (con tienda)</t>
+        </is>
+      </c>
+      <c r="F45" s="3" t="inlineStr">
+        <is>
+          <t>vía web</t>
+        </is>
+      </c>
+      <c r="G45" s="19" t="inlineStr">
+        <is>
+          <t>6618-0279; michvallar@lefleurbymichellevallarino.com</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="inlineStr">
+        <is>
+          <t>Michelle Vallarino</t>
+        </is>
+      </c>
+      <c r="I45" s="3" t="inlineStr">
+        <is>
+          <t>Tienda online; reseñas en opinamos.io</t>
+        </is>
+      </c>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="K45" s="3" t="inlineStr">
+        <is>
+          <t>Una floristería con e-commerce que además decora bodas: los pedidos chicos y las bodas de 15 mil entran por el mismo chat sin prioridad.</t>
+        </is>
+      </c>
+      <c r="L45" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M45" s="7" t="n"/>
+      <c r="N45" s="6" t="n"/>
+      <c r="O45" s="6" t="n"/>
+      <c r="P45" s="6" t="n"/>
+    </row>
+    <row r="46" ht="84" customHeight="1">
+      <c r="A46" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Bodas y eventos</t>
+        </is>
+      </c>
+      <c r="C46" s="6" t="inlineStr">
+        <is>
+          <t>2 · Fácil</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>Casa Casco (rooftop y salones, Plaza Herrera)</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>casacasco.com</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>vía web</t>
+        </is>
+      </c>
+      <c r="G46" s="19" t="inlineStr">
+        <is>
+          <t>WhatsApp 6288-9024; reservas 6136-8700; eventos@guamholding.com</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr">
+        <is>
+          <t>Guam Holding (grupo local)</t>
+        </is>
+      </c>
+      <c r="I46" s="3" t="inlineStr">
+        <is>
+          <t>WhatsApp dedicado a eventos</t>
+        </is>
+      </c>
+      <c r="J46" s="3" t="inlineStr">
+        <is>
+          <t>Venue icónico del Casco</t>
+        </is>
+      </c>
+      <c r="K46" s="3" t="inlineStr">
+        <is>
+          <t>Un rooftop del Casco recibe la misma pregunta 50 veces al mes: capacidad, mínimo de consumo, fecha. Eso lo responde un asistente y deja al equipo solo las visitas.</t>
+        </is>
+      </c>
+      <c r="L46" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M46" s="7" t="n"/>
+      <c r="N46" s="6" t="n"/>
+      <c r="O46" s="6" t="n"/>
+      <c r="P46" s="6" t="n"/>
+    </row>
+    <row r="47" ht="84" customHeight="1">
+      <c r="A47" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="B47" s="3" t="inlineStr">
+        <is>
+          <t>Agentes y alquiler corto</t>
+        </is>
+      </c>
+      <c r="C47" s="6" t="inlineStr">
+        <is>
+          <t>2 · Fácil</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>Estela's Realty Services · agente dueña de firma</t>
+        </is>
+      </c>
+      <c r="E47" s="5" t="inlineStr">
+        <is>
+          <t>estelasrealty.com</t>
+        </is>
+      </c>
+      <c r="F47" s="3" t="inlineStr">
+        <is>
+          <t>@estelasrealtyservices</t>
+        </is>
+      </c>
+      <c r="G47" s="19" t="inlineStr">
+        <is>
+          <t>+507 6612-9836 (PTY) / 6675-1521 (Boquete)</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="inlineStr">
+        <is>
+          <t>Estela (fundadora, desde 1981)</t>
+        </is>
+      </c>
+      <c r="I47" s="3" t="inlineStr">
+        <is>
+          <t>11 páginas de listados en encuentra24 (pauta premium)</t>
+        </is>
+      </c>
+      <c r="J47" s="3" t="inlineStr">
+        <is>
+          <t>38+ años; también administración y trámites</t>
+        </is>
+      </c>
+      <c r="K47" s="3" t="inlineStr">
+        <is>
+          <t>Con 11 páginas de anuncios en encuentra24, el cuello de botella no es el tráfico: es quién contesta y da seguimiento a cada consulta repetida.</t>
+        </is>
+      </c>
+      <c r="L47" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M47" s="7" t="n"/>
+      <c r="N47" s="6" t="n"/>
+      <c r="O47" s="6" t="n"/>
+      <c r="P47" s="6" t="n"/>
+    </row>
+    <row r="48" ht="84" customHeight="1">
+      <c r="A48" s="3" t="n">
+        <v>47</v>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Agentes y alquiler corto</t>
+        </is>
+      </c>
+      <c r="C48" s="6" t="inlineStr">
+        <is>
+          <t>2 · Fácil</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>Panama Property Guru · bróker individual (expats)</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>panamapropertyguru.com</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>@panamapropertyguru (2.4K)</t>
+        </is>
+      </c>
+      <c r="G48" s="19" t="inlineStr">
+        <is>
+          <t>+507 6151-8248 (WA)</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
+        <is>
+          <t>No nombrado</t>
+        </is>
+      </c>
+      <c r="I48" s="3" t="inlineStr">
+        <is>
+          <t>WordPress con membresía de pago; YouTube</t>
+        </is>
+      </c>
+      <c r="J48" s="3" t="inlineStr">
+        <is>
+          <t>Enfoque relocation</t>
+        </is>
+      </c>
+      <c r="K48" s="3" t="inlineStr">
+        <is>
+          <t>Sus leads son expats en otro huso horario: la mitad escribe cuando usted duerme y el competidor que responde primero se lleva la visita.</t>
+        </is>
+      </c>
+      <c r="L48" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M48" s="7" t="n"/>
+      <c r="N48" s="6" t="n"/>
+      <c r="O48" s="6" t="n"/>
+      <c r="P48" s="6" t="n"/>
+    </row>
+    <row r="49" ht="84" customHeight="1">
+      <c r="A49" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="B49" s="3" t="inlineStr">
+        <is>
+          <t>Agentes y alquiler corto</t>
+        </is>
+      </c>
+      <c r="C49" s="6" t="inlineStr">
+        <is>
+          <t>2 · Fácil</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>Nuba Rentals (Playa Venao) · administradora</t>
+        </is>
+      </c>
+      <c r="E49" s="5" t="inlineStr">
+        <is>
+          <t>nuba.rentals</t>
+        </is>
+      </c>
+      <c r="F49" s="3" t="inlineStr">
+        <is>
+          <t>@nubarentals</t>
+        </is>
+      </c>
+      <c r="G49" s="19" t="inlineStr">
+        <is>
+          <t>+507 6200-2788; reservations@nuba.rentals</t>
+        </is>
+      </c>
+      <c r="H49" s="3" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="I49" s="3" t="inlineStr">
+        <is>
+          <t>Airbnb, Booking, Expedia, VRBO + directas</t>
+        </is>
+      </c>
+      <c r="J49" s="3" t="inlineStr">
+        <is>
+          <t>Villas premium US$500+/noche</t>
+        </is>
+      </c>
+      <c r="K49" s="3" t="inlineStr">
+        <is>
+          <t>Sus villas de 500 dólares la noche reciben preguntas de grupos que comparan tres destinos a la vez: el que confirma disponibilidad en dos minutos gana la reserva.</t>
+        </is>
+      </c>
+      <c r="L49" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M49" s="7" t="n"/>
+      <c r="N49" s="6" t="n"/>
+      <c r="O49" s="6" t="n"/>
+      <c r="P49" s="6" t="n"/>
+    </row>
+    <row r="50" ht="84" customHeight="1">
+      <c r="A50" s="3" t="n">
+        <v>49</v>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Agentes y alquiler corto</t>
+        </is>
+      </c>
+      <c r="C50" s="6" t="inlineStr">
+        <is>
+          <t>2 · Fácil</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>Over The Water Rentals (Bocas) · administradores</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>overthewaterrentals.com</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G50" s="19" t="inlineStr">
+        <is>
+          <t>+507 6401-9021 (WA); 757-9516</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr">
+        <is>
+          <t>Claudia y Marlin</t>
+        </is>
+      </c>
+      <c r="I50" s="3" t="inlineStr">
+        <is>
+          <t>Airbnb desde 2010, TripAdvisor</t>
+        </is>
+      </c>
+      <c r="J50" s="3" t="inlineStr">
+        <is>
+          <t>Superhost 6 años; 6 casas sobre el agua</t>
+        </is>
+      </c>
+      <c r="K50" s="3" t="inlineStr">
+        <is>
+          <t>Seis años de Superhost y las reservas siguen dependiendo de que Claudia o Marlin vean el teléfono.</t>
+        </is>
+      </c>
+      <c r="L50" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M50" s="7" t="n"/>
+      <c r="N50" s="6" t="n"/>
+      <c r="O50" s="6" t="n"/>
+      <c r="P50" s="6" t="n"/>
+    </row>
+    <row r="51" ht="84" customHeight="1">
+      <c r="A51" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="B51" s="3" t="inlineStr">
+        <is>
+          <t>Agentes y alquiler corto</t>
+        </is>
+      </c>
+      <c r="C51" s="6" t="inlineStr">
+        <is>
+          <t>2 · Fácil</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>Boquete Vacation Rentals (JJM Inversiones) · administradora</t>
+        </is>
+      </c>
+      <c r="E51" s="5" t="inlineStr">
+        <is>
+          <t>boquetevacations.com (Squarespace)</t>
+        </is>
+      </c>
+      <c r="F51" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G51" s="19" t="inlineStr">
+        <is>
+          <t>+507 6660-0034; boquetevacations@gmail.com</t>
+        </is>
+      </c>
+      <c r="H51" s="3" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="I51" s="3" t="inlineStr">
+        <is>
+          <t>Web bilingüe; 'full service property management'</t>
+        </is>
+      </c>
+      <c r="J51" s="3" t="inlineStr">
+        <is>
+          <t>~8 unidades; 20 años</t>
+        </is>
+      </c>
+      <c r="K51" s="3" t="inlineStr">
+        <is>
+          <t>Boquete solo tiene 47 permisos de alquiler vacacional; usted tiene la oferta escasa, pero las consultas en inglés y español llegan al mismo celular sin filtro.</t>
+        </is>
+      </c>
+      <c r="L51" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M51" s="7" t="n"/>
+      <c r="N51" s="6" t="n"/>
+      <c r="O51" s="6" t="n"/>
+      <c r="P51" s="6" t="n"/>
+    </row>
+    <row r="52" ht="84" customHeight="1">
+      <c r="A52" s="3" t="n">
+        <v>51</v>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Agentes y alquiler corto</t>
+        </is>
+      </c>
+      <c r="C52" s="6" t="inlineStr">
+        <is>
+          <t>2 · Fácil</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>Panama Beach View (Tammy, Coronado Bay) · administradora</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>panamabeachview.com</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G52" s="19" t="inlineStr">
+        <is>
+          <t>+507 6529-2688 (WA)</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr">
+        <is>
+          <t>Tammy</t>
+        </is>
+      </c>
+      <c r="I52" s="3" t="inlineStr">
+        <is>
+          <t>Airbnb (Superhost)</t>
+        </is>
+      </c>
+      <c r="J52" s="3" t="inlineStr">
+        <is>
+          <t>~3 condos + casa</t>
+        </is>
+      </c>
+      <c r="K52" s="3" t="inlineStr">
+        <is>
+          <t>Sus tarifas semanales y mensuales dependen de que Tammy conteste cada WhatsApp; un asistente cotiza, confirma fechas y manda el link de pago.</t>
+        </is>
+      </c>
+      <c r="L52" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M52" s="7" t="n"/>
+      <c r="N52" s="6" t="n"/>
+      <c r="O52" s="6" t="n"/>
+      <c r="P52" s="6" t="n"/>
+    </row>
+    <row r="53" ht="84" customHeight="1">
+      <c r="A53" s="3" t="n">
+        <v>52</v>
+      </c>
+      <c r="B53" s="3" t="inlineStr">
+        <is>
+          <t>Autos seminuevos premium</t>
+        </is>
+      </c>
+      <c r="C53" s="20" t="inlineStr">
+        <is>
+          <t>3 · Después</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>@autodolarpty (solo Instagram)</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>sin web</t>
+        </is>
+      </c>
+      <c r="F53" s="3" t="inlineStr">
+        <is>
+          <t>@autodolarpty (49K)</t>
+        </is>
+      </c>
+      <c r="G53" s="19" t="inlineStr">
+        <is>
+          <t>Número en el botón de la bio (no visible en búsqueda)</t>
+        </is>
+      </c>
+      <c r="H53" s="3" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="I53" s="3" t="inlineStr">
+        <is>
+          <t>Bio: compra, venta, trade-in, avalúos gratis, 'escríbenos al WhatsApp'</t>
+        </is>
+      </c>
+      <c r="J53" s="3" t="inlineStr">
+        <is>
+          <t>49K seguidores, 1,941 posts</t>
+        </is>
+      </c>
+      <c r="K53" s="3" t="inlineStr">
+        <is>
+          <t>Todo su negocio vive en un botón de WhatsApp de Instagram; sin web, sin seguimiento, sin memoria de quién preguntó por qué carro.</t>
+        </is>
+      </c>
+      <c r="L53" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M53" s="7" t="n"/>
+      <c r="N53" s="6" t="n"/>
+      <c r="O53" s="6" t="n"/>
+      <c r="P53" s="6" t="n"/>
+    </row>
+    <row r="54" ht="84" customHeight="1">
+      <c r="A54" s="3" t="n">
+        <v>53</v>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Mejoras del hogar (alto ticket)</t>
+        </is>
+      </c>
+      <c r="C54" s="20" t="inlineStr">
+        <is>
+          <t>3 · Después</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>Piscinas Neptuno (fibra de vidrio, fábrica en Chame)</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>sin web propia clara</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>@piscinas_neptuno (190)</t>
+        </is>
+      </c>
+      <c r="G54" s="19" t="inlineStr">
+        <is>
+          <t>+507 6337-5365</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="I54" s="3" t="inlineStr">
+        <is>
+          <t>Visitas a fábrica con cita; directorios</t>
+        </is>
+      </c>
+      <c r="J54" s="3" t="inlineStr">
+        <is>
+          <t>Garantía 5 años; entrega 2-6 semanas</t>
+        </is>
+      </c>
+      <c r="K54" s="3" t="inlineStr">
+        <is>
+          <t>Fabrican piscinas de 15 mil con garantía de 5 años y solo tienen 190 seguidores: el producto vende, pero nadie lo ve ni lo agenda sin llamar.</t>
+        </is>
+      </c>
+      <c r="L54" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M54" s="7" t="n"/>
+      <c r="N54" s="6" t="n"/>
+      <c r="O54" s="6" t="n"/>
+      <c r="P54" s="6" t="n"/>
+    </row>
+    <row r="55" ht="84" customHeight="1">
+      <c r="A55" s="3" t="n">
+        <v>54</v>
+      </c>
+      <c r="B55" s="3" t="inlineStr">
+        <is>
+          <t>Mejoras del hogar (alto ticket)</t>
+        </is>
+      </c>
+      <c r="C55" s="20" t="inlineStr">
+        <is>
+          <t>3 · Después</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>24clima (aire acondicionado premium)</t>
+        </is>
+      </c>
+      <c r="E55" s="5" t="inlineStr">
+        <is>
+          <t>24clima.com</t>
+        </is>
+      </c>
+      <c r="F55" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G55" s="19" t="inlineStr">
+        <is>
+          <t>+507 6828-2120</t>
+        </is>
+      </c>
+      <c r="H55" s="3" t="inlineStr">
+        <is>
+          <t>Dueño HVAC master formado en Alemania</t>
+        </is>
+      </c>
+      <c r="I55" s="3" t="inlineStr">
+        <is>
+          <t>Ya venden 'respuesta en menos de 2 h'; español, inglés y ruso</t>
+        </is>
+      </c>
+      <c r="J55" s="3" t="inlineStr">
+        <is>
+          <t>Google 5.0 (11 reseñas); 9+ años</t>
+        </is>
+      </c>
+      <c r="K55" s="3" t="inlineStr">
+        <is>
+          <t>Prometen respuesta en menos de dos horas con un equipo humano: un asistente 24/7 convierte esa promesa en segundos sin contratar a nadie.</t>
+        </is>
+      </c>
+      <c r="L55" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M55" s="7" t="n"/>
+      <c r="N55" s="6" t="n"/>
+      <c r="O55" s="6" t="n"/>
+      <c r="P55" s="6" t="n"/>
+    </row>
+    <row r="56" ht="84" customHeight="1">
+      <c r="A56" s="3" t="n">
+        <v>55</v>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Instaladores solares</t>
+        </is>
+      </c>
+      <c r="C56" s="20" t="inlineStr">
+        <is>
+          <t>3 · Después</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>Solaris Energy (Azuero, expats)</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>solaris-panama.com</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G56" s="19" t="inlineStr">
+        <is>
+          <t>+507 6583-1822</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="I56" s="3" t="inlineStr">
+        <is>
+          <t>CTA 'envía tu ubicación y factura por WhatsApp'; web en inglés</t>
+        </is>
+      </c>
+      <c r="J56" s="3" t="inlineStr">
+        <is>
+          <t>Expats Pedasí/Azuero</t>
+        </is>
+      </c>
+      <c r="K56" s="3" t="inlineStr">
+        <is>
+          <t>Todo entra por WhatsApp en inglés y lo contesta una persona: la IA bilingüe califica y agenda sin que el dueño deje la instalación.</t>
+        </is>
+      </c>
+      <c r="L56" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M56" s="7" t="n"/>
+      <c r="N56" s="6" t="n"/>
+      <c r="O56" s="6" t="n"/>
+      <c r="P56" s="6" t="n"/>
+    </row>
+    <row r="57" ht="84" customHeight="1">
+      <c r="A57" s="3" t="n">
+        <v>56</v>
+      </c>
+      <c r="B57" s="3" t="inlineStr">
+        <is>
+          <t>Instaladores solares</t>
+        </is>
+      </c>
+      <c r="C57" s="20" t="inlineStr">
+        <is>
+          <t>3 · Después</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>Energy and Solar Solutions (familia Neblett)</t>
+        </is>
+      </c>
+      <c r="E57" s="5" t="inlineStr">
+        <is>
+          <t>energyandsolarsolutions.com</t>
+        </is>
+      </c>
+      <c r="F57" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="G57" s="19" t="inlineStr">
+        <is>
+          <t>Tel +507 374-1725 (fijo, sin WhatsApp visible)</t>
+        </is>
+      </c>
+      <c r="H57" s="3" t="inlineStr">
+        <is>
+          <t>David Neblett (CEO) y Daniel Neblett (director)</t>
+        </is>
+      </c>
+      <c r="I57" s="3" t="inlineStr">
+        <is>
+          <t>Perfil ENF, web propia</t>
+        </is>
+      </c>
+      <c r="J57" s="3" t="inlineStr">
+        <is>
+          <t>15+ años; baterías</t>
+        </is>
+      </c>
+      <c r="K57" s="3" t="inlineStr">
+        <is>
+          <t>Solo publican un fijo: el lead de Instagram no puede escribirles por WhatsApp y se va con el competidor.</t>
+        </is>
+      </c>
+      <c r="L57" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M57" s="7" t="n"/>
+      <c r="N57" s="6" t="n"/>
+      <c r="O57" s="6" t="n"/>
+      <c r="P57" s="6" t="n"/>
+    </row>
+    <row r="58" ht="84" customHeight="1">
+      <c r="A58" s="3" t="n">
+        <v>57</v>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>Bodas y eventos</t>
+        </is>
+      </c>
+      <c r="C58" s="20" t="inlineStr">
+        <is>
+          <t>3 · Después</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>Maito Catering (Grupo Maito, chef Mario Castrellón)</t>
+        </is>
+      </c>
+      <c r="E58" s="5" t="inlineStr">
+        <is>
+          <t>maitopanama.com/maito-catering</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>vía web</t>
+        </is>
+      </c>
+      <c r="G58" s="19" t="inlineStr">
+        <is>
+          <t>WhatsApp 6550-0377; 391-4657; info@maitopanama.com</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr">
+        <is>
+          <t>Mario Castrellón</t>
+        </is>
+      </c>
+      <c r="I58" s="3" t="inlineStr">
+        <is>
+          <t>Prensa internacional (50 Best)</t>
+        </is>
+      </c>
+      <c r="J58" s="3" t="inlineStr">
+        <is>
+          <t>Maito en Latin America's 50 Best</t>
+        </is>
+      </c>
+      <c r="K58" s="3" t="inlineStr">
+        <is>
+          <t>La marca más fuerte del país en gastronomía recibe pedidos de boda por el mismo WhatsApp que las reservas del restaurante; una degustación se puede agendar sola.</t>
+        </is>
+      </c>
+      <c r="L58" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M58" s="7" t="n"/>
+      <c r="N58" s="6" t="n"/>
+      <c r="O58" s="6" t="n"/>
+      <c r="P58" s="6" t="n"/>
+    </row>
+    <row r="59" ht="84" customHeight="1">
+      <c r="A59" s="3" t="n">
+        <v>58</v>
+      </c>
+      <c r="B59" s="3" t="inlineStr">
+        <is>
+          <t>Bodas y eventos</t>
+        </is>
+      </c>
+      <c r="C59" s="20" t="inlineStr">
+        <is>
+          <t>3 · Después</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>Lala Event Designers (planner de lujo)</t>
+        </is>
+      </c>
+      <c r="E59" s="5" t="inlineStr">
+        <is>
+          <t>lalapanama.com</t>
+        </is>
+      </c>
+      <c r="F59" s="3" t="inlineStr">
+        <is>
+          <t>@lalaeventdesigners (23K)</t>
+        </is>
+      </c>
+      <c r="G59" s="19" t="inlineStr">
+        <is>
+          <t>6179-1753; hola@lalapanama.com</t>
+        </is>
+      </c>
+      <c r="H59" s="3" t="inlineStr">
+        <is>
+          <t>Jess (y Sebas)</t>
+        </is>
+      </c>
+      <c r="I59" s="3" t="inlineStr">
+        <is>
+          <t>'VOGUE certified', Latin American Wedding Awards, bodas destino</t>
+        </is>
+      </c>
+      <c r="J59" s="3" t="inlineStr">
+        <is>
+          <t>8+ años</t>
+        </is>
+      </c>
+      <c r="K59" s="3" t="inlineStr">
+        <is>
+          <t>Con 23K seguidores, el DM se llena de '¿precio?'; nadie filtra fecha, invitados y presupuesto antes de que Jess conteste a mano. Entrar después de tener dos casos locales.</t>
+        </is>
+      </c>
+      <c r="L59" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M59" s="7" t="n"/>
+      <c r="N59" s="6" t="n"/>
+      <c r="O59" s="6" t="n"/>
+      <c r="P59" s="6" t="n"/>
+    </row>
+    <row r="60" ht="84" customHeight="1">
+      <c r="A60" s="3" t="n">
+        <v>59</v>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>Bodas y eventos</t>
+        </is>
+      </c>
+      <c r="C60" s="20" t="inlineStr">
+        <is>
+          <t>3 · Después</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>Regina Events (bodas de lujo + catering)</t>
+        </is>
+      </c>
+      <c r="E60" s="5" t="inlineStr">
+        <is>
+          <t>reginaevent.com</t>
+        </is>
+      </c>
+      <c r="F60" s="3" t="inlineStr">
+        <is>
+          <t>@reginaevents (16K)</t>
+        </is>
+      </c>
+      <c r="G60" s="19" t="inlineStr">
+        <is>
+          <t>6925-2787; info@reginaevent.com</t>
+        </is>
+      </c>
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>Regina Ortiz (también dirige Prowep Academy)</t>
+        </is>
+      </c>
+      <c r="I60" s="3" t="inlineStr">
+        <is>
+          <t>Directorio pago bodas.com.mx; speaker internacional</t>
+        </is>
+      </c>
+      <c r="J60" s="3" t="inlineStr">
+        <is>
+          <t>Desde 2009; 200+ bodas</t>
+        </is>
+      </c>
+      <c r="K60" s="3" t="inlineStr">
+        <is>
+          <t>Regina da clases y conferencias; mientras está en escena, la novia que escribió a las 10 pm ya agendó visita con otro planner. Entrar después de tener dos casos locales.</t>
+        </is>
+      </c>
+      <c r="L60" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M60" s="7" t="n"/>
+      <c r="N60" s="6" t="n"/>
+      <c r="O60" s="6" t="n"/>
+      <c r="P60" s="6" t="n"/>
+    </row>
+    <row r="61" ht="84" customHeight="1">
+      <c r="A61" s="3" t="n">
+        <v>60</v>
+      </c>
+      <c r="B61" s="3" t="inlineStr">
+        <is>
+          <t>Agentes y alquiler corto</t>
+        </is>
+      </c>
+      <c r="C61" s="20" t="inlineStr">
+        <is>
+          <t>3 · Después</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>Realtor Panamá (@panamarealtor) · agente</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>sin web</t>
+        </is>
+      </c>
+      <c r="F61" s="3" t="inlineStr">
+        <is>
+          <t>@panamarealtor (2.3K)</t>
+        </is>
+      </c>
+      <c r="G61" s="19" t="inlineStr">
+        <is>
+          <t>+507 6149-1542</t>
+        </is>
+      </c>
+      <c r="H61" s="3" t="inlineStr">
+        <is>
+          <t>No identificado</t>
+        </is>
+      </c>
+      <c r="I61" s="3" t="inlineStr">
+        <is>
+          <t>IG como canal principal</t>
+        </is>
+      </c>
+      <c r="J61" s="3" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="K61" s="3" t="inlineStr">
+        <is>
+          <t>Todo su embudo vive en la bio de Instagram; una web de marca personal más un asistente convierte el DM en cita.</t>
+        </is>
+      </c>
+      <c r="L61" s="6" t="inlineStr">
+        <is>
+          <t>Pendiente</t>
+        </is>
+      </c>
+      <c r="M61" s="7" t="n"/>
+      <c r="N61" s="6" t="n"/>
+      <c r="O61" s="6" t="n"/>
+      <c r="P61" s="6" t="n"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:P61"/>
+  <dataValidations count="2">
+    <dataValidation sqref="L2:L61" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Pendiente,Investigado,Mockup hecho,Contactado,Respondió,Reunión,Cliente,Descartado"</formula1>
+    </dataValidation>
+    <dataValidation sqref="N2:N61" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Email,WhatsApp,LinkedIn,Instagram,Llamada,Presencial"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E3" r:id="rId2"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="rId3"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E9" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E10" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E11" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E12" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E13" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E15" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E16" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E17" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E18" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E19" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E24" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E25" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E27" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E28" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E29" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E30" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E31" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E32" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E33" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E35" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E36" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E37" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E38" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E42" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E60" r:id="rId54"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
@@ -4986,18 +9048,259 @@
         <v/>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" s="21" t="inlineStr">
+        <is>
+          <t>Prospectos fáciles (hoja Fáciles)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="11" t="inlineStr">
+        <is>
+          <t>Nicho</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>1 Muy fácil</t>
+        </is>
+      </c>
+      <c r="C16" s="11" t="inlineStr">
+        <is>
+          <t>2 Fácil</t>
+        </is>
+      </c>
+      <c r="D16" s="11" t="inlineStr">
+        <is>
+          <t>3 Después</t>
+        </is>
+      </c>
+      <c r="E16" s="11" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="F16" s="11" t="inlineStr">
+        <is>
+          <t>Contactados</t>
+        </is>
+      </c>
+      <c r="G16" s="11" t="inlineStr">
+        <is>
+          <t>Respondieron</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="12" t="inlineStr">
+        <is>
+          <t>Autos seminuevos premium</t>
+        </is>
+      </c>
+      <c r="B17" s="12">
+        <f>COUNTIFS(Fáciles!$B:$B,$A17,Fáciles!$C:$C,"1 · Muy fácil")</f>
+        <v/>
+      </c>
+      <c r="C17" s="12">
+        <f>COUNTIFS(Fáciles!$B:$B,$A17,Fáciles!$C:$C,"2 · Fácil")</f>
+        <v/>
+      </c>
+      <c r="D17" s="12">
+        <f>COUNTIFS(Fáciles!$B:$B,$A17,Fáciles!$C:$C,"3 · Después")</f>
+        <v/>
+      </c>
+      <c r="E17" s="12">
+        <f>SUM(B17:D17)</f>
+        <v/>
+      </c>
+      <c r="F17" s="12">
+        <f>COUNTIFS(Fáciles!$B:$B,$A17,Fáciles!$L:$L,"Contactado")+COUNTIFS(Fáciles!$B:$B,$A17,Fáciles!$L:$L,"Respondió")+COUNTIFS(Fáciles!$B:$B,$A17,Fáciles!$L:$L,"Reunión")+COUNTIFS(Fáciles!$B:$B,$A17,Fáciles!$L:$L,"Cliente")</f>
+        <v/>
+      </c>
+      <c r="G17" s="12">
+        <f>COUNTIFS(Fáciles!$B:$B,$A17,Fáciles!$L:$L,"Respondió")+COUNTIFS(Fáciles!$B:$B,$A17,Fáciles!$L:$L,"Reunión")+COUNTIFS(Fáciles!$B:$B,$A17,Fáciles!$L:$L,"Cliente")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="12" t="inlineStr">
+        <is>
+          <t>Mejoras del hogar (alto ticket)</t>
+        </is>
+      </c>
+      <c r="B18" s="12">
+        <f>COUNTIFS(Fáciles!$B:$B,$A18,Fáciles!$C:$C,"1 · Muy fácil")</f>
+        <v/>
+      </c>
+      <c r="C18" s="12">
+        <f>COUNTIFS(Fáciles!$B:$B,$A18,Fáciles!$C:$C,"2 · Fácil")</f>
+        <v/>
+      </c>
+      <c r="D18" s="12">
+        <f>COUNTIFS(Fáciles!$B:$B,$A18,Fáciles!$C:$C,"3 · Después")</f>
+        <v/>
+      </c>
+      <c r="E18" s="12">
+        <f>SUM(B18:D18)</f>
+        <v/>
+      </c>
+      <c r="F18" s="12">
+        <f>COUNTIFS(Fáciles!$B:$B,$A18,Fáciles!$L:$L,"Contactado")+COUNTIFS(Fáciles!$B:$B,$A18,Fáciles!$L:$L,"Respondió")+COUNTIFS(Fáciles!$B:$B,$A18,Fáciles!$L:$L,"Reunión")+COUNTIFS(Fáciles!$B:$B,$A18,Fáciles!$L:$L,"Cliente")</f>
+        <v/>
+      </c>
+      <c r="G18" s="12">
+        <f>COUNTIFS(Fáciles!$B:$B,$A18,Fáciles!$L:$L,"Respondió")+COUNTIFS(Fáciles!$B:$B,$A18,Fáciles!$L:$L,"Reunión")+COUNTIFS(Fáciles!$B:$B,$A18,Fáciles!$L:$L,"Cliente")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="12" t="inlineStr">
+        <is>
+          <t>Instaladores solares</t>
+        </is>
+      </c>
+      <c r="B19" s="12">
+        <f>COUNTIFS(Fáciles!$B:$B,$A19,Fáciles!$C:$C,"1 · Muy fácil")</f>
+        <v/>
+      </c>
+      <c r="C19" s="12">
+        <f>COUNTIFS(Fáciles!$B:$B,$A19,Fáciles!$C:$C,"2 · Fácil")</f>
+        <v/>
+      </c>
+      <c r="D19" s="12">
+        <f>COUNTIFS(Fáciles!$B:$B,$A19,Fáciles!$C:$C,"3 · Después")</f>
+        <v/>
+      </c>
+      <c r="E19" s="12">
+        <f>SUM(B19:D19)</f>
+        <v/>
+      </c>
+      <c r="F19" s="12">
+        <f>COUNTIFS(Fáciles!$B:$B,$A19,Fáciles!$L:$L,"Contactado")+COUNTIFS(Fáciles!$B:$B,$A19,Fáciles!$L:$L,"Respondió")+COUNTIFS(Fáciles!$B:$B,$A19,Fáciles!$L:$L,"Reunión")+COUNTIFS(Fáciles!$B:$B,$A19,Fáciles!$L:$L,"Cliente")</f>
+        <v/>
+      </c>
+      <c r="G19" s="12">
+        <f>COUNTIFS(Fáciles!$B:$B,$A19,Fáciles!$L:$L,"Respondió")+COUNTIFS(Fáciles!$B:$B,$A19,Fáciles!$L:$L,"Reunión")+COUNTIFS(Fáciles!$B:$B,$A19,Fáciles!$L:$L,"Cliente")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="12" t="inlineStr">
+        <is>
+          <t>Bodas y eventos</t>
+        </is>
+      </c>
+      <c r="B20" s="12">
+        <f>COUNTIFS(Fáciles!$B:$B,$A20,Fáciles!$C:$C,"1 · Muy fácil")</f>
+        <v/>
+      </c>
+      <c r="C20" s="12">
+        <f>COUNTIFS(Fáciles!$B:$B,$A20,Fáciles!$C:$C,"2 · Fácil")</f>
+        <v/>
+      </c>
+      <c r="D20" s="12">
+        <f>COUNTIFS(Fáciles!$B:$B,$A20,Fáciles!$C:$C,"3 · Después")</f>
+        <v/>
+      </c>
+      <c r="E20" s="12">
+        <f>SUM(B20:D20)</f>
+        <v/>
+      </c>
+      <c r="F20" s="12">
+        <f>COUNTIFS(Fáciles!$B:$B,$A20,Fáciles!$L:$L,"Contactado")+COUNTIFS(Fáciles!$B:$B,$A20,Fáciles!$L:$L,"Respondió")+COUNTIFS(Fáciles!$B:$B,$A20,Fáciles!$L:$L,"Reunión")+COUNTIFS(Fáciles!$B:$B,$A20,Fáciles!$L:$L,"Cliente")</f>
+        <v/>
+      </c>
+      <c r="G20" s="12">
+        <f>COUNTIFS(Fáciles!$B:$B,$A20,Fáciles!$L:$L,"Respondió")+COUNTIFS(Fáciles!$B:$B,$A20,Fáciles!$L:$L,"Reunión")+COUNTIFS(Fáciles!$B:$B,$A20,Fáciles!$L:$L,"Cliente")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="12" t="inlineStr">
+        <is>
+          <t>Agentes y alquiler corto</t>
+        </is>
+      </c>
+      <c r="B21" s="12">
+        <f>COUNTIFS(Fáciles!$B:$B,$A21,Fáciles!$C:$C,"1 · Muy fácil")</f>
+        <v/>
+      </c>
+      <c r="C21" s="12">
+        <f>COUNTIFS(Fáciles!$B:$B,$A21,Fáciles!$C:$C,"2 · Fácil")</f>
+        <v/>
+      </c>
+      <c r="D21" s="12">
+        <f>COUNTIFS(Fáciles!$B:$B,$A21,Fáciles!$C:$C,"3 · Después")</f>
+        <v/>
+      </c>
+      <c r="E21" s="12">
+        <f>SUM(B21:D21)</f>
+        <v/>
+      </c>
+      <c r="F21" s="12">
+        <f>COUNTIFS(Fáciles!$B:$B,$A21,Fáciles!$L:$L,"Contactado")+COUNTIFS(Fáciles!$B:$B,$A21,Fáciles!$L:$L,"Respondió")+COUNTIFS(Fáciles!$B:$B,$A21,Fáciles!$L:$L,"Reunión")+COUNTIFS(Fáciles!$B:$B,$A21,Fáciles!$L:$L,"Cliente")</f>
+        <v/>
+      </c>
+      <c r="G21" s="12">
+        <f>COUNTIFS(Fáciles!$B:$B,$A21,Fáciles!$L:$L,"Respondió")+COUNTIFS(Fáciles!$B:$B,$A21,Fáciles!$L:$L,"Reunión")+COUNTIFS(Fáciles!$B:$B,$A21,Fáciles!$L:$L,"Cliente")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="13" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B22" s="13">
+        <f>SUM(B17:B21)</f>
+        <v/>
+      </c>
+      <c r="C22" s="13">
+        <f>SUM(C17:C21)</f>
+        <v/>
+      </c>
+      <c r="D22" s="13">
+        <f>SUM(D17:D21)</f>
+        <v/>
+      </c>
+      <c r="E22" s="13">
+        <f>SUM(E17:E21)</f>
+        <v/>
+      </c>
+      <c r="F22" s="13">
+        <f>SUM(F17:F21)</f>
+        <v/>
+      </c>
+      <c r="G22" s="13">
+        <f>SUM(G17:G21)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="13" t="inlineStr">
+        <is>
+          <t>Tasa de respuesta</t>
+        </is>
+      </c>
+      <c r="B23" s="14">
+        <f>IF(F22=0,0,G22/F22)</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A29"/>
+  <dimension ref="A1:A35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="120" customWidth="1" min="1" max="1"/>
@@ -5186,6 +9489,41 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" s="17" t="inlineStr">
+        <is>
+          <t>Hoja 'Fáciles' (añadida el 4 de octubre)</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="16" t="inlineStr">
+        <is>
+          <t>Criterio de 'fácil': un solo dueño que decide, reachable por WhatsApp o Instagram, ya paga por leads (Instagram, encuentra24, SEO), ticket de US$2K a 80K por venta, y en su mayoría en Ciudad de Panamá para cerrar en persona.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="16" t="inlineStr">
+        <is>
+          <t>Para estos el producto principal es el asistente de WhatsApp (respuesta 24/7, calificación, agenda, seguimiento). La web es el complemento, no al revés.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="16" t="inlineStr">
+        <is>
+          <t>Facilidad 1 = escribir esta semana. 2 = escribir después de los 1. 3 = esperar a tener dos casos de éxito locales.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="16" t="inlineStr">
+        <is>
+          <t>Los números de WhatsApp vienen de bios, encuentra24 y webs; confirmar en el perfil antes del primer mensaje.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>